<commit_message>
Corrigida a comarca de 'São José do Egito'
</commit_message>
<xml_diff>
--- a/data/comarcas.xlsx
+++ b/data/comarcas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fortesefortes-my.sharepoint.com/personal/gabrieldesouza_fortesefortes_com_br/Documents/Documentos/GABRIEL/Processo_Cnj/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{13A19558-D6EF-419B-89A9-D44028F00E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F8ADF03-4BB4-4908-AE25-944E9C4DAC75}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="8_{13A19558-D6EF-419B-89A9-D44028F00E66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5BFAE3D-C76F-4788-9204-BD70272AC14F}"/>
   <bookViews>
-    <workbookView xWindow="-15480" yWindow="-1965" windowWidth="15600" windowHeight="18720" xr2:uid="{BE522FF7-EB00-4953-8763-7E308AD69858}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BE522FF7-EB00-4953-8763-7E308AD69858}"/>
   </bookViews>
   <sheets>
     <sheet name="Estados" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4056" uniqueCount="2142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4058" uniqueCount="2143">
   <si>
     <t xml:space="preserve">ESTADO </t>
   </si>
@@ -6466,6 +6466,9 @@
   </si>
   <si>
     <t>Tabira</t>
+  </si>
+  <si>
+    <t>São José do Egito</t>
   </si>
 </sst>
 </file>
@@ -6919,7 +6922,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26E15F5A-FB20-483C-855A-2FB0E34AF6D5}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G1888"/>
+  <dimension ref="A1:G1889"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" style="1" customWidth="1"/>
@@ -27702,6 +27705,17 @@
         <v>2141</v>
       </c>
     </row>
+    <row r="1889" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1889" s="1" t="s">
+        <v>1912</v>
+      </c>
+      <c r="B1889" s="10">
+        <v>3340</v>
+      </c>
+      <c r="C1889" s="1" t="s">
+        <v>2142</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1887" xr:uid="{26E15F5A-FB20-483C-855A-2FB0E34AF6D5}">
     <filterColumn colId="0">

</xml_diff>